<commit_message>
Submission package: Table 2/Figure 3 order (steroid glucuronides first), Figure 3 as 3+2 grid, sequential numbers in Figure 2a, criteria in Table 2 caption, Figure 4 caption trimmed; text v5.3 header, Table S3/S5 citations, justification of the high-vs-low control criterion
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WDn5T1yz4TRFaKpaKqad5Y
</commit_message>
<xml_diff>
--- a/submission_analytica/2_main_tables/Tables_main.xlsx
+++ b/submission_analytica/2_main_tables/Tables_main.xlsx
@@ -893,60 +893,60 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Biliverdin</t>
+          <t>Tetrahydrocortisone glucuronide (putative)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>BILIVERDIN</t>
+          <t>5.beta.-Pregnane-3.alpha.,17,21-triol-11,20-dione (tetrahydrocortisone; MS/MS of the co-eluting aglycone ion)</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>583.2553</v>
+        <v>558.2914</v>
       </c>
       <c r="E4" t="n">
-        <v>13.48</v>
+        <v>10.76</v>
       </c>
       <c r="F4" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>biliverdin IXα assumed; other IX isomers not resolved</t>
+          <t>tetrahydrocortisone/allo-tetrahydrocortisone and 3- vs 21-glucuronide not distinguished; a second isomer elutes at 11.06 min</t>
         </is>
       </c>
       <c r="J4" t="n">
-        <v>2.23</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2.4e-02</t>
+          <t>3.0e-02</t>
         </is>
       </c>
       <c r="L4" t="n">
-        <v>0.77</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>0.042</t>
+          <t>0.024</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>0.001</t>
+          <t>0.019</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>89/97/75</t>
+          <t>100/100/100</t>
         </is>
       </c>
     </row>
@@ -956,19 +956,19 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>LysoPC(16:0)</t>
+          <t>Biliverdin</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1-Palmitoyl-sn-glycero-3-phosphocholine</t>
+          <t>BILIVERDIN</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>496.3397</v>
+        <v>583.2553</v>
       </c>
       <c r="E5" t="n">
-        <v>16.71</v>
+        <v>13.48</v>
       </c>
       <c r="F5" t="n">
         <v>1</v>
@@ -983,33 +983,33 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>sn-1/sn-2 regioisomers not resolved</t>
+          <t>biliverdin IXα assumed; other IX isomers not resolved</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>1.33</v>
+        <v>2.23</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>2.5e-02</t>
+          <t>2.4e-02</t>
         </is>
       </c>
       <c r="L5" t="n">
-        <v>0.79</v>
+        <v>0.77</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>0.003</t>
+          <t>0.042</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>0.001</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>100/100/100</t>
+          <t>89/97/75</t>
         </is>
       </c>
     </row>
@@ -1019,55 +1019,55 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Tetrahydrocortisone glucuronide (putative)</t>
+          <t>LysoPC(16:0)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>5.beta.-Pregnane-3.alpha.,17,21-triol-11,20-dione (tetrahydrocortisone; MS/MS of the co-eluting aglycone ion)</t>
+          <t>1-Palmitoyl-sn-glycero-3-phosphocholine</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>558.2914</v>
+        <v>496.3397</v>
       </c>
       <c r="E6" t="n">
-        <v>10.76</v>
+        <v>16.71</v>
       </c>
       <c r="F6" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>tetrahydrocortisone/allo-tetrahydrocortisone and 3- vs 21-glucuronide not distinguished; a second isomer elutes at 11.06 min</t>
+          <t>sn-1/sn-2 regioisomers not resolved</t>
         </is>
       </c>
       <c r="J6" t="n">
-        <v>0.8100000000000001</v>
+        <v>1.33</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>3.0e-02</t>
+          <t>2.5e-02</t>
         </is>
       </c>
       <c r="L6" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.79</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>0.024</t>
+          <t>0.003</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>0.019</t>
+          <t>0.000</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -1087,7 +1087,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Isomers: 11-Oxoetiocholanolone glucuronide (putative): 11-oxoetiocholanolone and 11-oxoandrosterone glucuronides (5β/5α) not distinguished; identity assigned from the aglycone MS/MS; Tetrahydrocortisone glucuronide (putative): tetrahydrocortisone/allo-tetrahydrocortisone and 3- vs 21-glucuronide not distinguished; a second isomer elutes at 10.76 min; Biliverdin: biliverdin IXα assumed; other IX isomers not resolved; LysoPC(16:0): sn-1/sn-2 regioisomers not resolved; Tetrahydrocortisone glucuronide (putative): tetrahydrocortisone/allo-tetrahydrocortisone and 3- vs 21-glucuronide not distinguished; a second isomer elutes at 11.06 min</t>
+          <t>Isomers: 11-Oxoetiocholanolone glucuronide (putative): 11-oxoetiocholanolone and 11-oxoandrosterone glucuronides (5β/5α) not distinguished; identity assigned from the aglycone MS/MS; Tetrahydrocortisone glucuronide (putative): tetrahydrocortisone/allo-tetrahydrocortisone and 3- vs 21-glucuronide not distinguished; a second isomer elutes at 10.76 min; Tetrahydrocortisone glucuronide (putative): tetrahydrocortisone/allo-tetrahydrocortisone and 3- vs 21-glucuronide not distinguished; a second isomer elutes at 11.06 min; Biliverdin: biliverdin IXα assumed; other IX isomers not resolved; LysoPC(16:0): sn-1/sn-2 regioisomers not resolved</t>
         </is>
       </c>
     </row>

</xml_diff>